<commit_message>
fix(privacy): redact surviving bit serials, add serial-number rule
Real equipment serial numbers survived the first M43 pass: as text in three
DDR evidence JSONs and as numeric cells (DDR Data!N52:N53) in the shipped
cell dump and the de-identified fixture. Text is replaced by
[REDACTED:serial]; numeric cells are overwritten with synthetic values by the
existing sanitizer (fixture re-pinned). Digests join the denylist and a new
equipment-serial-number rule has synthetic positive/negative tests.

The purge plan now records a verified full-history inventory (17 blobs,
300 of 454 commits), a blob substitution for the zipped fixture, and that
the default branch still serves the real workbook (owner containment step).

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/synthetic_ddr_golden_a.xlsx
+++ b/tests/fixtures/synthetic_ddr_golden_a.xlsx
@@ -23021,7 +23021,7 @@
       </c>
       <c r="M52" s="1038"/>
       <c r="N52" s="1038">
-        <v>1515041004</v>
+        <v>1000000001</v>
       </c>
       <c r="O52" s="1038"/>
       <c r="P52" s="1039">
@@ -23061,7 +23061,7 @@
       </c>
       <c r="M53" s="1038"/>
       <c r="N53" s="1038">
-        <v>15013006</v>
+        <v>10000002</v>
       </c>
       <c r="O53" s="1038"/>
       <c r="P53" s="1039">

</xml_diff>